<commit_message>
PAUSED: checkpoint, task198 re-rooted to a verdict and five builders live
task198 architecture 3 assigned: the same world, pack and variance component
with the decision moved from a pick of one region to a characterisation of one
named region's move, which is what the variance rule filed in stumping Part 3
licenses. Guard run before briefing: structural_verdict with shape 18 returns
PASS with no BLOCK and no WARN, and the new driver sits 0.07 from its nearest
neighbour on file while architecture 2's own driver is outside the top eight.

In flight here: task194's final confirmation run and its card brought up to
architecture 3, task196's prompt gate at 982 characters with the estimator
forms its judge asked for now asserted, task197 with precut at 50 of 50 and
its remaining gates running.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017NMcBvUc2Vu9DKDdwmhqo4
</commit_message>
<xml_diff>
--- a/task196/golden/member_incidence_review.xlsx
+++ b/task196/golden/member_incidence_review.xlsx
@@ -532,13 +532,13 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>22301200</v>
+        <v>22233300</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>400</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F2" t="n">
         <v>31</v>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -716,7 +716,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -819,13 +819,13 @@
         <v>311088</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>272896</v>
+        <v>271791</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>81499</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>665484</v>
+        <v>664379</v>
       </c>
     </row>
     <row r="3">
@@ -838,13 +838,13 @@
         <v>309882</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>230899</v>
+        <v>228966</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>83191</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>623972</v>
+        <v>622039</v>
       </c>
     </row>
     <row r="4">
@@ -857,13 +857,13 @@
         <v>317029</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>220954</v>
+        <v>222673</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>75171</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>613153</v>
+        <v>614872</v>
       </c>
     </row>
     <row r="5">
@@ -876,13 +876,13 @@
         <v>339633</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>182147</v>
+        <v>181104</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>75823</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>597604</v>
+        <v>596560</v>
       </c>
     </row>
   </sheetData>
@@ -928,10 +928,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>322554</v>
+        <v>307226</v>
       </c>
     </row>
     <row r="3">
@@ -1126,13 +1126,13 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>5.7</v>
+        <v>6.5</v>
       </c>
       <c r="C2" s="4" t="n">
-        <v>4.4</v>
+        <v>3.4</v>
       </c>
       <c r="D2" s="4" t="n">
-        <v>2.3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="3">
@@ -1142,13 +1142,13 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>12.9</v>
+        <v>15.1</v>
       </c>
       <c r="C3" s="4" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="D3" s="4" t="n">
         <v>3.8</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="4">
@@ -1158,13 +1158,13 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>5.8</v>
+        <v>8.5</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>7.4</v>
+        <v>2.5</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>0.9</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="5">
@@ -1174,13 +1174,13 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>8.699999999999999</v>
+        <v>5.4</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>5.1</v>
+        <v>2.5</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>3.7</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="6">
@@ -1190,13 +1190,13 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>7.9</v>
+        <v>8.5</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>5.4</v>
+        <v>2.7</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2.3</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>